<commit_message>
Updated CHN model - 2025-09-20 19:30
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{352508FC-F5ED-47F7-A530-F94EA04EC362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F7AE6B6-2BCA-4555-9E29-525C2BB9366A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8184,7 +8184,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D5E4C0B-8E9B-4A92-8BB1-E6D786379A88}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27E45554-5C90-4C88-976F-68A07D79C223}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12997,7 +12997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3E10B50-3F14-4729-B749-CBA984C49B16}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D2B2097-071E-4AFB-89E3-8AEB92B7FD27}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18201,7 +18201,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EDC0C24-4D85-4ECD-9FF3-9B39AB414A7B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19044F5A-00B8-4C29-9D99-BF140908D818}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-09-20 19:36
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F7AE6B6-2BCA-4555-9E29-525C2BB9366A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE8EA1DF-AFBE-4B3F-8AA6-FF921F5C680C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8184,7 +8184,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27E45554-5C90-4C88-976F-68A07D79C223}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA6A096-CFF9-4B38-82F5-03844D37AD9B}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12997,7 +12997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D2B2097-071E-4AFB-89E3-8AEB92B7FD27}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FFFE725-7A5E-405F-B323-4F92649362DF}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18201,7 +18201,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19044F5A-00B8-4C29-9D99-BF140908D818}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{843C4ABB-6A14-4255-B820-71F1573BE24C}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-09-20 20:02
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE8EA1DF-AFBE-4B3F-8AA6-FF921F5C680C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CED2041-C7DD-4AB2-82FD-E607662972E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8184,7 +8184,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA6A096-CFF9-4B38-82F5-03844D37AD9B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52016D2F-3146-4FC2-BCD0-A890B6F0B1D6}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12997,7 +12997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FFFE725-7A5E-405F-B323-4F92649362DF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E516BBD-CDEC-4864-9C96-E832F97834B8}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18201,7 +18201,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{843C4ABB-6A14-4255-B820-71F1573BE24C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9D35A2-3C81-4A11-A966-C82BC1E324CA}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-09-23 10:50
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3705C7D8-8227-4445-AD25-6D8ECAB5324B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D6B862-8534-4519-8ACE-9BD07A707364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72596C3-38EE-4195-B8F9-823E8476E027}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8E83BFB-8390-4E79-8D11-028217DF7411}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6545392-DC4E-427F-93F2-6CB925EE9A40}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886C200B-4253-4A9E-9168-AE3E38208631}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10724901-D199-41A7-9CE3-FAC6DC16E215}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F6155E5-1F3C-4F3B-96AC-ED599E469913}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-09-23 15:30
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D6B862-8534-4519-8ACE-9BD07A707364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{36E6FBF9-44AE-4515-AFCA-4C9B9DEB7AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8E83BFB-8390-4E79-8D11-028217DF7411}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C896C4DC-466B-46C5-ACAC-9F7BC8ECFD41}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886C200B-4253-4A9E-9168-AE3E38208631}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD555617-4CD3-4DE4-A9E3-CF155C12F7D6}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F6155E5-1F3C-4F3B-96AC-ED599E469913}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB40048-AC9C-4368-8750-0A1F817E024D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 13:25
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5B69633-C6A0-4435-916F-A62E64EE98C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A022711-56C8-4E9B-B131-2BACEEB85660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50AF16E3-1710-435F-8D16-96112F86222D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3BFD382-6AEA-4A13-9E49-CF2AE064BAC2}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEABED34-9C4D-4891-A9E4-FE6250814ED0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C474B3-D42F-4727-909B-4FCAEEF059AD}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC9A66A-7441-45F4-871B-0F33069D4555}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28086F5E-4BD6-4EB0-A2A2-52DCD188D92D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 13:36
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A022711-56C8-4E9B-B131-2BACEEB85660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{831759D6-4F7E-42C0-B375-FEB2B7FC7F52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3BFD382-6AEA-4A13-9E49-CF2AE064BAC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B76C81CA-B903-4111-8637-A73CC402A159}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C474B3-D42F-4727-909B-4FCAEEF059AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84FB5A2-02E5-4B73-9692-A1A85C00F762}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28086F5E-4BD6-4EB0-A2A2-52DCD188D92D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8EDAA3A-D671-4C92-9FE6-D246E164EE11}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 13:48
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{831759D6-4F7E-42C0-B375-FEB2B7FC7F52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0B219A1-25A8-4FBD-A8AB-3DC752F26DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B76C81CA-B903-4111-8637-A73CC402A159}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A80BCF1-2868-42C6-95FF-655EC6A84746}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84FB5A2-02E5-4B73-9692-A1A85C00F762}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD9BD2C-390B-4F2F-B1C7-324952C310DD}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8EDAA3A-D671-4C92-9FE6-D246E164EE11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87C40815-254D-48F7-A9A5-35887A96A901}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 14:13
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0B219A1-25A8-4FBD-A8AB-3DC752F26DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{212B6F8B-86D0-4759-99F9-C95F84326DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A80BCF1-2868-42C6-95FF-655EC6A84746}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74FE8B61-5493-413D-89F6-C683DBD15A69}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD9BD2C-390B-4F2F-B1C7-324952C310DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A0B75CC-A24D-435F-A2B0-D4429A870926}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87C40815-254D-48F7-A9A5-35887A96A901}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{907D1AEA-E8DA-4A8F-877A-7C4F3B6A13B0}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 14:23
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{212B6F8B-86D0-4759-99F9-C95F84326DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1652876D-8FFE-423F-B491-E14FFF860AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74FE8B61-5493-413D-89F6-C683DBD15A69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CDBFD6C-6110-4C08-A616-55E6A1FCE51F}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A0B75CC-A24D-435F-A2B0-D4429A870926}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C523C-2049-4A19-B35A-BC4B028B0FAB}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{907D1AEA-E8DA-4A8F-877A-7C4F3B6A13B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D21D5E5-D87E-4589-8A5E-B2F600205637}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 14:31
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1652876D-8FFE-423F-B491-E14FFF860AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC4B5D12-5E30-4FFF-AA49-08B0AF510921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CDBFD6C-6110-4C08-A616-55E6A1FCE51F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D94B013-0C20-4F1D-9E18-5CB9608BD1E1}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C523C-2049-4A19-B35A-BC4B028B0FAB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5D8651-76CD-4435-8B7C-0EAB93467884}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D21D5E5-D87E-4589-8A5E-B2F600205637}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4606B4CD-B721-43C8-BEBA-6FC0DEC3DDC8}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN model - 2025-10-31 14:43
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CHN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC4B5D12-5E30-4FFF-AA49-08B0AF510921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BC1782D-D7E7-4F60-8173-E975FA8418AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8001,7 +8001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D94B013-0C20-4F1D-9E18-5CB9608BD1E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A36C151-F787-40CE-BCF8-CB95BF650C10}">
   <dimension ref="B9:M146"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12814,7 +12814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5D8651-76CD-4435-8B7C-0EAB93467884}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F33FFD4-0C49-4DD2-86FB-2C4B55098DC9}">
   <dimension ref="B9:Z124"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18018,7 +18018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4606B4CD-B721-43C8-BEBA-6FC0DEC3DDC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D03314-6A9D-43DB-8380-94B2AAB9E1C6}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>